<commit_message>
feat: menus personalizados en tabla con hoja oculta menu_list_app, multiples correos Outlook, eliminacion fisica y limpieza PDF de plantillas Word, proyecto Formatos Lector Tutor y unificacion Iniciar_Correspon.bat
</commit_message>
<xml_diff>
--- a/Proyectos_Correspondencia/Titulacion/Titulacion_Matriz.xlsx
+++ b/Proyectos_Correspondencia/Titulacion/Titulacion_Matriz.xlsx
@@ -406,8 +406,16 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025-1</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>